<commit_message>
Improve clarity in workshop4 Sections 4 and 8: standardize pNP naming and ANOVA object names
</commit_message>
<xml_diff>
--- a/raw-data/BIO00066I-pNP-example-data-2025-26.xlsx
+++ b/raw-data/BIO00066I-pNP-example-data-2025-26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dj757/Library/CloudStorage/GoogleDrive-daniel.jeffares@york.ac.uk/My Drive/modules/BIO66I/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C2B56DB-F970-EC4B-96B7-C29ABDEE9114}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7F751854-FAB9-BA48-B636-E7EAB0228DE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="50360" windowHeight="24680" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="50360" windowHeight="24680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="standard curve" sheetId="1" r:id="rId1"/>

</xml_diff>